<commit_message>
Add 5-year periods and ETS/NETS
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_SYS_CarbonBudget-CAP24_400MT-new.xlsx
+++ b/SuppXLS/Scen_SYS_CarbonBudget-CAP24_400MT-new.xlsx
@@ -1,24 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SuppXLS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BSuleimenov\Documents\GitHub\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C856AEC-59DA-4D6E-87BB-D92927C0EFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA1284B-F773-42EB-80AE-D2A500B738B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="24" r:id="rId1"/>
     <sheet name="Regions" sheetId="15" r:id="rId2"/>
     <sheet name="config" sheetId="20" r:id="rId3"/>
     <sheet name="single" sheetId="21" r:id="rId4"/>
-    <sheet name="multi" sheetId="22" r:id="rId5"/>
-    <sheet name="negative_CO2" sheetId="23" r:id="rId6"/>
+    <sheet name="negative_CO2" sheetId="23" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="__123Graph_AEUMILKPN" localSheetId="0" hidden="1">#REF!</definedName>
@@ -140,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="121">
   <si>
     <t>LimType</t>
   </si>
@@ -360,12 +359,6 @@
     <t>UC_RHSR</t>
   </si>
   <si>
-    <t>UC - All Regions/Each Period</t>
-  </si>
-  <si>
-    <t>UC_RHS</t>
-  </si>
-  <si>
     <t>UC_desc</t>
   </si>
   <si>
@@ -522,13 +515,13 @@
     <t>COM_CUMNET</t>
   </si>
   <si>
-    <t>UC_Sets: T_S:</t>
-  </si>
-  <si>
     <t>2021-2030</t>
   </si>
   <si>
-    <t>2021-2050</t>
+    <t>Bakytzhan Suleimenov (UCC, bsuleimenov@ucc.ie)</t>
+  </si>
+  <si>
+    <t>2021-2051</t>
   </si>
 </sst>
 </file>
@@ -5396,7 +5389,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>19050</xdr:colOff>
+          <xdr:colOff>22860</xdr:colOff>
           <xdr:row>3</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -5784,17 +5777,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43ACE639-45BB-4BC0-8EFB-335579A1276F}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" customWidth="1"/>
-    <col min="8" max="10" width="8.140625" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" customWidth="1"/>
-    <col min="12" max="12" width="8.140625" customWidth="1"/>
+    <col min="1" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" customWidth="1"/>
+    <col min="8" max="10" width="8.109375" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" customWidth="1"/>
+    <col min="12" max="12" width="8.109375" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" customWidth="1"/>
-    <col min="15" max="15" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" customWidth="1"/>
+    <col min="15" max="15" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -6219,7 +6212,7 @@
     </row>
     <row r="16" spans="1:26" ht="102.75" customHeight="1">
       <c r="A16" s="42" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B16" s="42"/>
       <c r="C16" s="42"/>
@@ -6305,10 +6298,10 @@
     </row>
     <row r="19" spans="1:26" ht="17.25" customHeight="1">
       <c r="A19" s="25" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B19" s="41" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C19" s="41"/>
       <c r="D19" s="41"/>
@@ -6337,10 +6330,10 @@
     </row>
     <row r="20" spans="1:26" ht="17.25" customHeight="1">
       <c r="A20" s="25" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B20" s="41" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C20" s="41"/>
       <c r="D20" s="41"/>
@@ -6369,10 +6362,10 @@
     </row>
     <row r="21" spans="1:26" ht="17.25" customHeight="1">
       <c r="A21" s="25" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C21" s="28"/>
       <c r="D21" s="28"/>
@@ -6429,10 +6422,10 @@
     </row>
     <row r="23" spans="1:26" ht="17.25" customHeight="1">
       <c r="A23" s="25" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B23" s="41" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C23" s="41"/>
       <c r="D23" s="41"/>
@@ -6517,10 +6510,10 @@
     </row>
     <row r="26" spans="1:26" ht="17.25" customHeight="1">
       <c r="A26" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" s="41" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="C26" s="41"/>
       <c r="D26" s="41"/>
@@ -6605,7 +6598,7 @@
     </row>
     <row r="29" spans="1:26" ht="17.25" customHeight="1">
       <c r="A29" s="25" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B29" s="29"/>
       <c r="C29" s="28"/>
@@ -6635,10 +6628,10 @@
     </row>
     <row r="30" spans="1:26" ht="17.25" customHeight="1">
       <c r="A30" s="25" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B30" s="43" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C30" s="41"/>
       <c r="D30" s="41"/>
@@ -6667,10 +6660,10 @@
     </row>
     <row r="31" spans="1:26" ht="17.25" customHeight="1">
       <c r="A31" s="25" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B31" s="41" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C31" s="41"/>
       <c r="D31" s="41"/>
@@ -6700,7 +6693,7 @@
     <row r="32" spans="1:26" ht="17.25" customHeight="1">
       <c r="A32" s="31"/>
       <c r="B32" s="32" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C32" s="31"/>
       <c r="D32" s="31"/>
@@ -8627,36 +8620,36 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42C030FF-C503-4743-9DBD-437AEB1E949D}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A3:AD37"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.5703125" customWidth="1"/>
-    <col min="25" max="25" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="3" max="3" width="3.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.5546875" customWidth="1"/>
+    <col min="25" max="25" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.109375" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:30">
@@ -9127,7 +9120,7 @@
         <v>IE-MN</v>
       </c>
     </row>
-    <row r="10" spans="1:30" ht="15.75" thickBot="1">
+    <row r="10" spans="1:30" ht="15" thickBot="1">
       <c r="A10" s="3" t="s">
         <v>32</v>
       </c>
@@ -9369,7 +9362,7 @@
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>19050</xdr:colOff>
+                    <xdr:colOff>22860</xdr:colOff>
                     <xdr:row>3</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -9388,14 +9381,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011941A8-04BF-45E8-9F60-D4E07475AB4A}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B4:G26"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9405,7 +9398,7 @@
       </c>
       <c r="C4" t="str">
         <f xml:space="preserve"> _xlfn.TEXTJOIN("_",TRUE,"UC","CB",ROUND(C7,0),"Mt",C6)</f>
-        <v>UC_CB_400_Mt_2021-2050</v>
+        <v>UC_CB_400_Mt_2021-2051</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" ref="D4:E4" si="0" xml:space="preserve"> _xlfn.TEXTJOIN("_",TRUE,"UC","CB",ROUND(D7,0),"Mt",D6)</f>
@@ -9422,11 +9415,11 @@
     </row>
     <row r="5" spans="2:6">
       <c r="B5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C5" t="str">
         <f xml:space="preserve"> _xlfn.TEXTJOIN(" ",TRUE,"Carbon budget",ROUND(C7,0),"Mt",C6)</f>
-        <v>Carbon budget 400 Mt 2021-2050</v>
+        <v>Carbon budget 400 Mt 2021-2051</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" ref="D5:F5" si="2" xml:space="preserve"> _xlfn.TEXTJOIN(" ",TRUE,"Carbon budget",ROUND(D7,0),"Mt",D6)</f>
@@ -9443,24 +9436,24 @@
     </row>
     <row r="6" spans="2:6">
       <c r="B6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C7" s="17">
         <f>D19</f>
@@ -9480,19 +9473,19 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="2:6">
@@ -9500,50 +9493,50 @@
         <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="2:6">
       <c r="B10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="2:6">
@@ -9551,21 +9544,21 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="2:6">
       <c r="B13" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C13">
         <v>-1</v>
@@ -9582,7 +9575,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -9602,7 +9595,7 @@
     </row>
     <row r="19" spans="3:7">
       <c r="C19" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D19" s="35">
         <v>400</v>
@@ -9610,29 +9603,29 @@
     </row>
     <row r="22" spans="3:7">
       <c r="C22" s="33" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="3:7">
       <c r="C23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D23" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E23" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="E23" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="F23" s="34" t="s">
-        <v>107</v>
-      </c>
       <c r="G23" s="34" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="3:7">
       <c r="C24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D24" s="34">
         <f>40+54+29+7+30+5.2</f>
@@ -9652,7 +9645,7 @@
     </row>
     <row r="26" spans="3:7">
       <c r="C26" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -9666,20 +9659,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9318C9B-7F0A-410C-BCB5-F22D93E1F454}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:L14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -9689,13 +9682,13 @@
     </row>
     <row r="2" spans="1:12">
       <c r="B2" s="9" t="str">
-        <f>"~UC_Sets: R_E: "  &amp; _xlfn.TEXTJOIN(",",TRUE,Regions!C3)</f>
-        <v>~UC_Sets: R_E: IE</v>
+        <f>"~UC_Sets: R_S:"</f>
+        <v>~UC_Sets: R_S:</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="B3" s="9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -9712,25 +9705,25 @@
         <v>62</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>0</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K5" s="8" t="s">
         <v>65</v>
@@ -9741,7 +9734,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="B6" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -9752,14 +9745,14 @@
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L6" s="13"/>
     </row>
     <row r="7" spans="1:12">
       <c r="B7" t="str">
         <f>VLOOKUP($B$5, config!$B$4:$F$14,2,FALSE) &amp; "_Single"</f>
-        <v>UC_CB_400_Mt_2021-2050_Single</v>
+        <v>UC_CB_400_Mt_2021-2051_Single</v>
       </c>
       <c r="C7" t="str">
         <f>VLOOKUP(C$5, config!$B$4:$F$14,2,FALSE)</f>
@@ -9771,7 +9764,7 @@
       </c>
       <c r="F7" t="str">
         <f>VLOOKUP(F$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>2021-2050</v>
+        <v>2021-2051</v>
       </c>
       <c r="G7" t="str">
         <f>VLOOKUP(G$5, config!$B$4:$F$14,2,FALSE)</f>
@@ -9791,223 +9784,7 @@
       </c>
       <c r="L7" t="str">
         <f>VLOOKUP($L$5, config!$B$4:$F$14,2,FALSE) &amp; " - Single"</f>
-        <v>Carbon budget 400 Mt 2021-2050 - Single</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="B8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D8" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E8" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F8" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>2021-2050</v>
-      </c>
-      <c r="J8">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>-1</v>
-      </c>
-      <c r="K8" s="17"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="B9" t="str">
-        <f>"\I:"&amp;VLOOKUP($B$5, config!$B$4:$F$14,3,FALSE) &amp; "_Single"</f>
-        <v>\I:UC_CB_274_Mt_2021-2030_Single</v>
-      </c>
-      <c r="C9" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D9" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F9" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>2021-2030</v>
-      </c>
-      <c r="G9" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H9" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I9">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K9" s="17">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,3,FALSE)*1000</f>
-        <v>274200</v>
-      </c>
-      <c r="L9" t="str">
-        <f>VLOOKUP($L$5, config!$B$4:$F$14,3,FALSE) &amp; " - Single"</f>
-        <v>Carbon budget 274 Mt 2021-2030 - Single</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="B10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C10" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D10" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E10" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F10" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>2021-2030</v>
-      </c>
-      <c r="J10">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>-1</v>
-      </c>
-      <c r="K10" s="17"/>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="B11" t="str">
-        <f>"\I:"&amp;VLOOKUP($B$5, config!$B$4:$F$14,4,FALSE) &amp; "_Single"</f>
-        <v>\I:UC_CB_126_Mt_2031-2050_Single</v>
-      </c>
-      <c r="C11" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D11" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F11" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>2031-2050</v>
-      </c>
-      <c r="G11" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H11" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I11">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K11" s="17">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,4,FALSE)*1000</f>
-        <v>125800.00000000001</v>
-      </c>
-      <c r="L11" t="str">
-        <f>VLOOKUP($L$5, config!$B$4:$F$14,4,FALSE) &amp; " - Single"</f>
-        <v>Carbon budget 126 Mt 2031-2050 - Single</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="B12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C12" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D12" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E12" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F12" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>2031-2050</v>
-      </c>
-      <c r="J12">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="B13" t="str">
-        <f>VLOOKUP($B$5, config!$B$4:$F$14,5,FALSE) &amp; "_Single"</f>
-        <v>UC_CB_0_Mt_2051-2100_Single</v>
-      </c>
-      <c r="C13" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D13" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F13" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>2051-2100</v>
-      </c>
-      <c r="G13" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H13" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I13">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K13">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,5,FALSE)*1000</f>
-        <v>0</v>
-      </c>
-      <c r="L13" t="str">
-        <f>VLOOKUP($L$5, config!$B$4:$F$14,5,FALSE) &amp; " - Single"</f>
-        <v>Carbon budget 0 Mt 2051-2100 - Single</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="B14" t="s">
-        <v>112</v>
-      </c>
-      <c r="C14" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D14" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E14" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F14" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>2051-2100</v>
-      </c>
-      <c r="J14">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>-1</v>
+        <v>Carbon budget 400 Mt 2021-2051 - Single</v>
       </c>
     </row>
   </sheetData>
@@ -10017,388 +9794,34 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6EC2971-91FC-4261-B0BB-58C7F43C1746}">
-  <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:L14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
-  <cols>
-    <col min="2" max="2" width="33.140625" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="33.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="B2" s="9" t="str">
-        <f>"UC_Sets: R_S: " &amp; _xlfn.TEXTJOIN(",",TRUE,Regions!D3:AD3)</f>
-        <v xml:space="preserve">UC_Sets: R_S: </v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="B3" s="9" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="H4" t="str">
-        <f>IF(RIGHT(B2,1)&lt;&gt;" ","UC_T","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="B5" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="L5" s="10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="B6" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="L6" s="7"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="B7" t="str">
-        <f>VLOOKUP(B$5, config!$B$4:$F$14,2,FALSE) &amp; "_Multi"</f>
-        <v>UC_CB_400_Mt_2021-2050_Multi</v>
-      </c>
-      <c r="C7" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D7" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F7" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>2021-2050</v>
-      </c>
-      <c r="G7" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H7" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I7">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K7" s="17">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,2,FALSE)*1000</f>
-        <v>400000</v>
-      </c>
-      <c r="L7" t="str">
-        <f>VLOOKUP(L$5, config!$B$4:$F$14,2,FALSE) &amp; " - Multi"</f>
-        <v>Carbon budget 400 Mt 2021-2050 - Multi</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="B8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D8" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E8" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F8" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>2021-2050</v>
-      </c>
-      <c r="J8">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,2,FALSE)</f>
-        <v>-1</v>
-      </c>
-      <c r="K8" s="17"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="B9" t="str">
-        <f>VLOOKUP(B$5, config!$B$4:$F$14,3,FALSE) &amp; "_Multi"</f>
-        <v>UC_CB_274_Mt_2021-2030_Multi</v>
-      </c>
-      <c r="C9" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D9" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F9" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>2021-2030</v>
-      </c>
-      <c r="G9" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H9" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I9">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K9" s="17">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,3,FALSE)*1000</f>
-        <v>274200</v>
-      </c>
-      <c r="L9" t="str">
-        <f>VLOOKUP(L$5, config!$B$4:$F$14,3,FALSE) &amp; " - Multi"</f>
-        <v>Carbon budget 274 Mt 2021-2030 - Multi</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="B10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C10" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D10" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E10" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F10" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>2021-2030</v>
-      </c>
-      <c r="J10">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,3,FALSE)</f>
-        <v>-1</v>
-      </c>
-      <c r="K10" s="17"/>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="B11" t="str">
-        <f>"\I:"&amp;VLOOKUP(B$5, config!$B$4:$F$14,4,FALSE) &amp; "_Multi"</f>
-        <v>\I:UC_CB_126_Mt_2031-2050_Multi</v>
-      </c>
-      <c r="C11" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D11" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F11" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>2031-2050</v>
-      </c>
-      <c r="G11" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H11" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I11">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K11" s="17">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,4,FALSE)*1000</f>
-        <v>125800.00000000001</v>
-      </c>
-      <c r="L11" t="str">
-        <f>VLOOKUP(L$5, config!$B$4:$F$14,4,FALSE) &amp; " - Multi"</f>
-        <v>Carbon budget 126 Mt 2031-2050 - Multi</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="B12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C12" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D12" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E12" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F12" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>2031-2050</v>
-      </c>
-      <c r="J12">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,4,FALSE)</f>
-        <v>-1</v>
-      </c>
-      <c r="K12" s="17"/>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="B13" t="str">
-        <f>VLOOKUP(B$5, config!$B$4:$F$14,5,FALSE) &amp; "_Multi"</f>
-        <v>UC_CB_0_Mt_2051-2100_Multi</v>
-      </c>
-      <c r="C13" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D13" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="F13" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>2051-2100</v>
-      </c>
-      <c r="G13" t="str">
-        <f>VLOOKUP(G$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>NET</v>
-      </c>
-      <c r="H13" t="str">
-        <f>VLOOKUP(H$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>UP</v>
-      </c>
-      <c r="I13">
-        <f>VLOOKUP(I$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="K13" s="17">
-        <f>VLOOKUP("Value", config!$B$4:$F$14,5,FALSE)*1000</f>
-        <v>0</v>
-      </c>
-      <c r="L13" t="str">
-        <f>VLOOKUP(L$5, config!$B$4:$F$14,5,FALSE) &amp; " - Multi"</f>
-        <v>Carbon budget 0 Mt 2051-2100 - Multi</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="B14" t="s">
-        <v>112</v>
-      </c>
-      <c r="C14" t="str">
-        <f>VLOOKUP(C$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>TOTCO2</v>
-      </c>
-      <c r="D14" t="str">
-        <f>VLOOKUP(D$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>ENV</v>
-      </c>
-      <c r="E14" t="str">
-        <f>VLOOKUP(E$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>T-A*INT*,T-NAV*</v>
-      </c>
-      <c r="F14" t="str">
-        <f>VLOOKUP(F$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>2051-2100</v>
-      </c>
-      <c r="J14">
-        <f>VLOOKUP(J$5, config!$B$4:$F$14,5,FALSE)</f>
-        <v>-1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2314F01-B0DB-448B-9217-DEB90E2D1CCA}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="B2:I12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9">
       <c r="B2" s="14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" ht="15.75" thickBot="1">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" ht="15" thickBot="1">
       <c r="B3" s="15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C3" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F3" s="15" t="s">
         <v>62</v>
@@ -10414,16 +9837,16 @@
     </row>
     <row r="4" spans="2:9">
       <c r="C4" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G4" s="17">
         <v>-1</v>
@@ -10435,7 +9858,7 @@
     </row>
     <row r="7" spans="2:9">
       <c r="B7" s="38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D7" s="36"/>
       <c r="E7" s="36"/>
@@ -10444,27 +9867,27 @@
       <c r="H7" s="36"/>
       <c r="I7" s="36"/>
     </row>
-    <row r="8" spans="2:9" ht="15.75" thickBot="1">
+    <row r="8" spans="2:9" ht="15" thickBot="1">
       <c r="B8" s="39" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C8" s="39" t="s">
         <v>0</v>
       </c>
       <c r="D8" s="39" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E8" s="39" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G8" s="39" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H8" s="39" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I8" s="39" t="s">
         <v>62</v>
@@ -10472,10 +9895,10 @@
     </row>
     <row r="9" spans="2:9">
       <c r="C9" s="36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E9" s="36">
         <v>0</v>
@@ -10486,15 +9909,15 @@
       <c r="G9" s="36"/>
       <c r="H9" s="36"/>
       <c r="I9" s="37" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="2:9">
       <c r="C10" s="36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E10" s="36"/>
       <c r="F10" s="40">
@@ -10503,18 +9926,18 @@
       <c r="G10" s="36"/>
       <c r="H10" s="36"/>
       <c r="I10" s="37" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="2:9">
       <c r="B11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E11" s="36">
         <v>0</v>
@@ -10525,15 +9948,15 @@
       <c r="G11" s="36"/>
       <c r="H11" s="36"/>
       <c r="I11" s="37" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="2:9">
       <c r="C12" s="36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E12" s="36"/>
       <c r="F12" s="40">
@@ -10542,7 +9965,7 @@
       <c r="G12" s="36"/>
       <c r="H12" s="36"/>
       <c r="I12" s="37" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>